<commit_message>
Exploratory work moves to the private repository: workflows write there, monthly feed-screen spreadsheet
Author's decision, 31 Oct 2026: every sweep in addition to the core (data, analysis and
reports) goes to the private repository pagagne/snapshot-manual. Feed screen, Honeypot capture
and the exploratory Research tasks save there through tools/private.sh and print counts only;
Manual publish keeps exploratory/ and runs/ there and rebuilds Part III from them; Backup copies
the private repository to Drive. New: snapshot.feedsheet (clickable titles, abstract and key
findings as pop-up notes), made by every feed screen. One-off Private move workflow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ja62sVwuRgkZ7eiKHxiFMr
</commit_message>
<xml_diff>
--- a/exploratory/feed-screen-2026-10.xlsx
+++ b/exploratory/feed-screen-2026-10.xlsx
@@ -1113,7 +1113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="390">
   <si>
     <t xml:space="preserve">Read one item</t>
   </si>
@@ -1151,13 +1151,13 @@
     <t xml:space="preserve">How to use</t>
   </si>
   <si>
-    <t xml:space="preserve">Type an item number in the yellow cell B3; the item's details appear above. Click the title to open the article.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On the Feed sweep tab, hover over any title to see its abstract and key findings in a pop-up note; click the title to open the article.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decision colours: green = logged as a new case; yellow = your judgement; blue = second source; grey = already logged; white = excluded.</t>
+    <t xml:space="preserve">Type an item number in the yellow cell B3; its details appear above. Click the title to open the article.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On the Feed sweep tab, rest the pointer on any title to see its abstract and key findings in a pop-up note; click the title to open the article.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision colours: green = logged as a new case; yellow = your judgement; blue = second source; grey = already logged; white = excluded or not yet sorted.</t>
   </si>
   <si>
     <t xml:space="preserve">'Summary based on': 'Report read by Claude' means Claude read the organisation's report; 'Title and feed entry' means the summary comes from the title, the feed entry and the screen only.</t>
@@ -2330,6 +2330,9 @@
   </si>
   <si>
     <t xml:space="preserve">Items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not yet sorted</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -2374,15 +2377,15 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
-      <color rgb="FF0000FF"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2513,12 +2516,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2917,7 +2920,7 @@
   <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
   </cols>
   <sheetData>
@@ -2927,98 +2930,96 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>10</v>
+      <c r="B3" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$B$2:$B$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>2026-10-29</v>
+        <v>2026-10-30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$C$2:$C$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>CrowdStrike</v>
+        <v>SecurityLab (ru)</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">IFERROR(HYPERLINK(INDEX(Links!$B$2:$B$66,MATCH($B$3,Links!$A$2:$A$66,0)),INDEX('Feed sweep'!$D$2:$D$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0))),"")</f>
-        <v>VAPOR PANDA Uses AI-Driven ARTEX to Scale a Global Espionage Campaign</v>
+        <v>Binance взломали. С крупнейшей криптобиржи вывели почти $6 млрд за час</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$E$2:$E$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>CrowdStrike reports that the China-nexus group VAPOR PANDA ran ARTEX AI agents (planner and worker agents) in a global espionage campaign from 17 Oct.</v>
+        <v>Russian news digest led by a theft of almost $6 billion from the Binance exchange in an hour.</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$F$2:$F$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>200+ organisations targeted in at least 14 countries; post-exploitation confirmed at 9.
-Targets: foreign ministries, government, semiconductors, defence, nuclear, finance, telecoms.
-Open-weight models named; single source so far. New log row.</v>
+        <v>No sign the attacker used AI; excluded from the AI-attack log.</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$G$2:$G$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>logged</v>
+        <v>excluded</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$H$2:$H$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>VAPOR PANDA (CrowdStrike); new log row; single source, large scale</v>
+        <v>no AI use by the attacker in the report (crypto exchange and wallet thefts, Linux kernel flaw, routing abuse, product statistics, VMmanager attack, BEC, ASOS breach); matched only on general AI words</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="5" t="str">
         <f aca="false">IFERROR(IF(INDEX('Feed sweep'!$I$2:$I$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0))="","(none)",HYPERLINK(INDEX('Feed sweep'!$I$2:$I$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),INDEX('Feed sweep'!$I$2:$I$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)))),"")</f>
-        <v>https://www.crowdstrike.com/en-us/blog/vapor-panda-uses-artex-to-scale-global-campaign/</v>
+        <v>(none)</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feed sweep'!$J$2:$J$66,MATCH($B$3,'Feed sweep'!$A$2:$A$66,0)),"")</f>
-        <v>Report read by Claude</v>
+        <v>Title and feed entry</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -5644,10 +5645,10 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="12" t="s">
         <v>328</v>
       </c>
     </row>
@@ -6187,7 +6188,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -6206,7 +6207,7 @@
         <v>82</v>
       </c>
       <c r="B2" s="14" t="n">
-        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,A2)</f>
+        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,"logged")</f>
         <v>9</v>
       </c>
     </row>
@@ -6215,7 +6216,7 @@
         <v>170</v>
       </c>
       <c r="B3" s="14" t="n">
-        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,A3)</f>
+        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,"second source")</f>
         <v>9</v>
       </c>
     </row>
@@ -6224,7 +6225,7 @@
         <v>210</v>
       </c>
       <c r="B4" s="14" t="n">
-        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,A4)</f>
+        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,"already logged")</f>
         <v>5</v>
       </c>
     </row>
@@ -6233,7 +6234,7 @@
         <v>52</v>
       </c>
       <c r="B5" s="14" t="n">
-        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,A5)</f>
+        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,"your judgement")</f>
         <v>6</v>
       </c>
     </row>
@@ -6242,16 +6243,25 @@
         <v>27</v>
       </c>
       <c r="B6" s="14" t="n">
-        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,A6)</f>
+        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,"excluded")</f>
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="14" t="s">
         <v>388</v>
       </c>
-      <c r="B7" s="3" t="n">
-        <f aca="false">SUM(B2:B6)</f>
+      <c r="B7" s="14" t="n">
+        <f aca="false">COUNTIF('Feed sweep'!$G$2:$G$66,"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <f aca="false">SUM(B2:B7)</f>
         <v>65</v>
       </c>
     </row>

</xml_diff>